<commit_message>
melhoria(visual): centraliza a imagem da logo entre as celulas F4 e G5
</commit_message>
<xml_diff>
--- a/modelo_relatorio.xlsx
+++ b/modelo_relatorio.xlsx
@@ -160,7 +160,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -234,11 +234,44 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <right/>
+      <top style="thin">
+        <color rgb="00E2E8F0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00E2E8F0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00E2E8F0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -404,6 +437,9 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -482,7 +518,6 @@
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -670,9 +705,9 @@
   <oneCellAnchor>
     <from>
       <col>5</col>
-      <colOff>0</colOff>
+      <colOff>504825</colOff>
       <row>3</row>
-      <rowOff>0</rowOff>
+      <rowOff>69818</rowOff>
     </from>
     <ext cx="1485900" cy="419100"/>
     <pic>
@@ -8412,7 +8447,6 @@
         <v/>
       </c>
     </row>
-    <row r="298"/>
     <row r="299">
       <c r="A299" s="15" t="n"/>
       <c r="B299" s="15" t="n"/>
@@ -8461,7 +8495,6 @@
       <c r="F301" s="6" t="n"/>
       <c r="G301" s="6" t="n"/>
     </row>
-    <row r="302"/>
     <row r="303">
       <c r="A303" s="20" t="inlineStr">
         <is>
@@ -8531,13 +8564,13 @@
           <t>CONSUMO TOTAL</t>
         </is>
       </c>
-      <c r="B5" s="39" t="n"/>
+      <c r="B5" s="61" t="n"/>
       <c r="C5" s="38" t="inlineStr">
         <is>
           <t>VALOR TOTAL RATEADO</t>
         </is>
       </c>
-      <c r="D5" s="39" t="n"/>
+      <c r="D5" s="61" t="n"/>
       <c r="E5" s="38" t="inlineStr">
         <is>
           <t>% TOP 10</t>
@@ -8548,24 +8581,24 @@
           <t>VARIAÇÃO GERAL VS MÉDIA</t>
         </is>
       </c>
-      <c r="G5" s="39" t="n"/>
+      <c r="G5" s="61" t="n"/>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="40" t="n">
         <v>689.0000000000001</v>
       </c>
-      <c r="B6" s="39" t="n"/>
+      <c r="B6" s="61" t="n"/>
       <c r="C6" s="41" t="n">
         <v>43875.52</v>
       </c>
-      <c r="D6" s="39" t="n"/>
+      <c r="D6" s="61" t="n"/>
       <c r="E6" s="42" t="n">
         <v>0.5766328011611029</v>
       </c>
       <c r="F6" s="43" t="n">
         <v>-0.1563985262852057</v>
       </c>
-      <c r="G6" s="39" t="n"/>
+      <c r="G6" s="61" t="n"/>
     </row>
     <row r="7" ht="10" customHeight="1"/>
     <row r="8" ht="26" customHeight="1">
@@ -8915,7 +8948,7 @@
       </c>
     </row>
     <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="58" t="inlineStr">
+      <c r="A23" s="62" t="inlineStr">
         <is>
           <t>Top 10 Maiores Consumidores</t>
         </is>
@@ -8926,7 +8959,7 @@
       </c>
     </row>
     <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="60" t="inlineStr">
+      <c r="A24" s="63" t="inlineStr">
         <is>
           <t>Demais Salas (279 un)</t>
         </is>

</xml_diff>